<commit_message>
feat: mid-month update Apr 2026 (through Apr 16)
Add April 2026 events scraped from status.fortify.com/history (BST->GMT converted):
- Apr 7: AMS Portal Service Degradation 18:03-19:21 GMT (excluded from uptime)
- Apr 8: FedRAMP Portal + API Outage 04:09-04:12 GMT (de-duped, 3 min)
- Apr 9: EU SAST Aviator Outage 19:11-19:13 GMT (2 min)
- Apr 9: EU SAST maintenance x2 windows
- Apr 10: AMS SAST maintenance 20:56-22:32 GMT
- Apr 11-16: no events

Apr partial: 2 outage incidents, 5 min. YTD (Jan-Mar completed): 14 incidents, 71 min, 99.9452%.

https://claude.ai/code/session_013wkzuwE47Hcmby5caq7Eqs
</commit_message>
<xml_diff>
--- a/FoD_Uptime_Report_2026.xlsx
+++ b/FoD_Uptime_Report_2026.xlsx
@@ -684,21 +684,21 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>2*</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>5*</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>0.0*</t>
+          <t>0.08*</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>1</v>
+        <v>0.9998842592592593</v>
       </c>
     </row>
     <row r="19">
@@ -2128,7 +2128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>100.0000%</t>
+          <t>99.9884%</t>
         </is>
       </c>
     </row>
@@ -2261,17 +2261,129 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>0.9979166666666667</v>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="12" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>0.9986111111111111</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Services Affected (to date)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Detailed Incidents (to date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>1. April 08, 2026 - Multiple Outages (3 minutes total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Service 1: Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Service 2: Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Time: 4:09 AM GMT-4:12 AM GMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Impact: Brief service disruption</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2. April 09, 2026 - Outage (2 minutes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Service: SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Time: 7:11 PM GMT-7:13 PM GMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Impact: Brief service disruption</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2337,21 +2449,21 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-10T20:56:00Z</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 10, 2026 10:32 PM GMT</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -2367,21 +2479,21 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-09T21:04:00Z</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 09, 2026 9:34 PM GMT</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -2392,30 +2504,30 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>203</v>
+        <v>2</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -2427,115 +2539,115 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-09T18:04:00Z</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 09, 2026 9:35 PM GMT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-08T04:10:00Z</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-08T04:09:00Z</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-07T18:03:00Z</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 07, 2026 7:21 PM GMT</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -2547,25 +2659,25 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -2577,25 +2689,25 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -2607,21 +2719,21 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>123</v>
+        <v>203</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -2637,21 +2749,21 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T21:04:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 10:34 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>90</v>
+        <v>203</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -2667,21 +2779,21 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T17:44:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 6:26 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>42</v>
+        <v>150</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -2697,21 +2809,21 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -2727,21 +2839,21 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -2752,26 +2864,26 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T00:43:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 12:46 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>3</v>
+        <v>123</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -2787,21 +2899,21 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>198</v>
+        <v>123</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -2817,21 +2929,21 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>198</v>
+        <v>123</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -2842,26 +2954,26 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T19:46:00Z</t>
+          <t>2026-03-20T21:04:00Z</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Mar 17, 2026 7:48 PM GMT</t>
+          <t>Mar 20, 2026 10:34 PM GMT</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -2872,26 +2984,26 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-03-13T00:37:00Z</t>
+          <t>2026-03-20T17:44:00Z</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Mar 13, 2026 12:41 AM GMT</t>
+          <t>Mar 20, 2026 6:26 PM GMT</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -2902,26 +3014,26 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-03-11T23:50:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Mar 11, 2026 11:54 PM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>4</v>
+        <v>99</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -2937,21 +3049,21 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>164</v>
+        <v>99</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -2962,26 +3074,26 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-18T00:43:00Z</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 18, 2026 12:46 AM GMT</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>164</v>
+        <v>3</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -2997,21 +3109,21 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>85</v>
+        <v>198</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -3027,21 +3139,21 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>85</v>
+        <v>198</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -3052,26 +3164,26 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-17T19:46:00Z</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 17, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -3082,26 +3194,26 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-13T00:37:00Z</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 13, 2026 12:41 AM GMT</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>87</v>
+        <v>4</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -3112,26 +3224,26 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-11T23:50:00Z</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 11, 2026 11:54 PM GMT</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -3147,21 +3259,21 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>95</v>
+        <v>164</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -3177,21 +3289,21 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>95</v>
+        <v>164</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -3207,21 +3319,21 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -3232,26 +3344,26 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 5:02 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -3262,26 +3374,26 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 4:56 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>5</v>
+        <v>87</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -3292,26 +3404,26 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:44:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 3:15 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -3322,26 +3434,26 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:42:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:44 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -3352,26 +3464,26 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:41:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:42 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
@@ -3382,30 +3494,30 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-02-26T16:39:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Feb 26, 2026 4:44 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -3417,115 +3529,115 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>207</v>
+        <v>95</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 02, 2026 5:02 PM GMT</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>207</v>
+        <v>11</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Mar 02, 2026 4:56 PM GMT</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-03-02T14:44:00Z</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Mar 02, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>159</v>
+        <v>31</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -3537,17 +3649,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2026-02-15T19:46:00Z</t>
+          <t>2026-03-02T14:42:00Z</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Feb 15, 2026 7:48 PM GMT</t>
+          <t>Mar 02, 2026 2:44 PM GMT</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
@@ -3555,7 +3667,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -3567,51 +3679,51 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14T22:07:00Z</t>
+          <t>2026-03-02T14:41:00Z</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Feb 14, 2026 10:09 PM GMT</t>
+          <t>Mar 02, 2026 2:42 PM GMT</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-26T16:39:00Z</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 26, 2026 4:44 PM GMT</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>282</v>
+        <v>5</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
@@ -3627,21 +3739,21 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>282</v>
+        <v>207</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
@@ -3657,21 +3769,21 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>127</v>
+        <v>207</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
@@ -3687,21 +3799,21 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
@@ -3717,21 +3829,21 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>98</v>
+        <v>159</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
@@ -3742,26 +3854,26 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-15T19:46:00Z</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 15, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
@@ -3772,26 +3884,26 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-14T22:07:00Z</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 14, 2026 10:09 PM GMT</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>88</v>
+        <v>2</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
@@ -3807,21 +3919,21 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>88</v>
+        <v>282</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
@@ -3837,25 +3949,25 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>4234</v>
+        <v>282</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -3867,72 +3979,72 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>4234</v>
+        <v>127</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:46:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:47 PM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>1</v>
+        <v>127</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:45:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:46 PM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -3941,11 +4053,11 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -3957,25 +4069,25 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>1595</v>
+        <v>98</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -3987,25 +4099,25 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>1595</v>
+        <v>88</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -4017,51 +4129,51 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T16:24:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Jan 20, 2026 3:26 AM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>4982</v>
+        <v>88</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T15:14:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:15 PM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>1</v>
+        <v>4234</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
@@ -4077,21 +4189,21 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T21:13:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:03 PM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>1070</v>
+        <v>4234</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
@@ -4107,17 +4219,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T04:24:00Z</t>
+          <t>2026-01-27T14:46:00Z</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Jan 15, 2026 4:25 AM GMT</t>
+          <t>Jan 27, 2026 2:47 PM GMT</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand - Vulncat</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">
@@ -4137,21 +4249,21 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>2026-01-10T15:08:00Z</t>
+          <t>2026-01-27T14:45:00Z</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Jan 10, 2026 3:10 PM GMT</t>
+          <t>Jan 27, 2026 2:46 PM GMT</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
@@ -4167,12 +4279,12 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -4181,7 +4293,7 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>140</v>
+        <v>1595</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
@@ -4197,12 +4309,12 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -4211,7 +4323,7 @@
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>140</v>
+        <v>1595</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
@@ -4227,21 +4339,21 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-16T16:24:00Z</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 20, 2026 3:26 AM GMT</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>137</v>
+        <v>4982</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
@@ -4252,26 +4364,26 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-16T15:14:00Z</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 16, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>137</v>
+        <v>1</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
@@ -4287,21 +4399,21 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T00:24:00Z</t>
+          <t>2026-01-15T21:13:00Z</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 1:02 AM GMT</t>
+          <t>Jan 16, 2026 3:03 PM GMT</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>38</v>
+        <v>1070</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
@@ -4312,37 +4424,247 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-15T04:24:00Z</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Jan 15, 2026 4:25 AM GMT</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand - Vulncat</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-10T15:08:00Z</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Jan 10, 2026 3:10 PM GMT</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T04:54:00Z</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T04:54:00Z</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - AMS</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>2026-01-08T00:24:00Z</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Jan 08, 2026 1:02 AM GMT</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T00:24:00Z</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 1:02 AM GMT</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
-      <c r="E68" s="5" t="n">
+      <c r="E75" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="F68" s="5" t="inlineStr">
+      <c r="F75" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>Report revised: April 04, 2026</t>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Report revised: April 16, 2026</t>
         </is>
       </c>
     </row>
@@ -4729,7 +5051,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Last updated: April 16, 2026 (mid-month update; April data through Apr 16, no new events since Apr 2).</t>
+          <t>Last updated: April 16, 2026 (mid-month update; April data through Apr 16; events added: Apr 7 AMS Portal degradation, Apr 8 FedRAMP outage 3 min, Apr 9 EU SAST outage 2 min, Apr 9-10 SAST maintenance windows).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: mid-month update May 2026 (through 2026-05-16)
May 1-16 events added:
- Outages (2): AMS SAST Aviator May 10 (2 min), EU SAST Aviator May 9 (2 min)
- Maintenance: APAC May 4, AMS May 8, SGP May 11-12
- Service Degradation (excluded): AMS May 7-8, AMS May 13

Back-fill: Apr 22 - May 4 AMS service degradation added to April data
(was in-progress at prior update, now complete; no impact on April uptime)

YTD unchanged: 18 outages, 96 min, 99.9444% (Jan-Apr completed months)
May partial: 2 outages, 4 min (not yet in YTD)
</commit_message>
<xml_diff>
--- a/FoD_Uptime_Report_2026.xlsx
+++ b/FoD_Uptime_Report_2026.xlsx
@@ -551,7 +551,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Completed Months: January - April 2026 (May in progress)</t>
+          <t>Completed Months: January - April 2026 (May in progress, partial through May 16)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -714,21 +714,21 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>2*</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>4*</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>0.0*</t>
+          <t>0.07*</t>
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>1</v>
+        <v>0.999910394265233</v>
       </c>
     </row>
     <row r="20">
@@ -942,7 +942,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>* May 2026 is in progress. Data will be finalized after May 31, 2026.</t>
+          <t>* May 2026 is in progress. Partial data through May 16, 2026. Will be finalized after May 31, 2026.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Last updated: May 2, 2026 (April finalized; April complete through Apr 30; events added Apr 17-30: AMS maintenance Apr 17-20, EU maintenance Apr 21-22, EMEA maintenance Apr 24, multi-region maintenance Apr 29-30; no new outages Apr 17-30).</t>
+          <t>Last updated: May 16, 2026 (mid-month snapshot through May 16; 2 outages added: AMS SAST Aviator May 10 2 min, EU SAST Aviator May 9 2 min; maintenance added: APAC May 4, AMS May 8, SGP May 11-12; service degradation events: AMS May 7-8 and May 13; Apr 22 - May 4 AMS service degradation back-filled to April data).</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Last updated: May 2, 2026</t>
+          <t>Last updated: May 16, 2026</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>1</v>
+        <v>0.9999551971326165</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
         <v>0.9999537037037037</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>1</v>
+        <v>0.9999551971326165</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -4500,7 +4500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4521,7 +4521,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Month in progress. To be finalized after May 31, 2026.</t>
+          <t>Month in progress. Partial data through May 16, 2026. To be finalized after May 31, 2026.</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>100.0000%</t>
+          <t>99.9910%</t>
         </is>
       </c>
     </row>
@@ -4633,17 +4633,115 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>0.9986111111111111</v>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="15" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>0.9986111111111111</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Services Affected (to date)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>SAST Aviator / ams-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Detailed Incidents (to date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>1. May 09, 2026 - Outage (2 minutes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Service: SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Time: 7:11 PM GMT-7:13 PM GMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Impact: Brief service disruption</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2. May 10, 2026 - Outage (2 minutes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Service: SAST Aviator / ams-sast-aviator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Time: 9:09 PM GMT-9:11 PM GMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Impact: Brief service disruption</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4704,17 +4802,17 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -4723,28 +4821,28 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>162</v>
+        <v>5</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -4753,11 +4851,11 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>162</v>
+        <v>5</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -4769,25 +4867,25 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>78</v>
+        <v>673</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -4799,85 +4897,85 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>78</v>
+        <v>673</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-05-10T21:09:00Z</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>May 10, 2026 9:11 PM GMT</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>88</v>
+        <v>2</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-05-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>May 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>88</v>
+        <v>2</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -4889,25 +4987,25 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>73</v>
+        <v>132</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -4919,85 +5017,85 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>73</v>
+        <v>132</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>273</v>
+        <v>1395</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>273</v>
+        <v>1395</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -5009,25 +5107,25 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>273</v>
+        <v>72</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -5039,25 +5137,25 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>273</v>
+        <v>72</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -5069,21 +5167,21 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>242</v>
+        <v>162</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -5099,21 +5197,21 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>242</v>
+        <v>162</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -5129,21 +5227,21 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1187</v>
+        <v>78</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -5159,21 +5257,21 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>1187</v>
+        <v>78</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -5189,21 +5287,21 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>4284</v>
+        <v>88</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -5219,21 +5317,21 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>4284</v>
+        <v>88</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -5244,26 +5342,26 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:28:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:38 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -5274,26 +5372,26 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:26:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:36 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -5309,21 +5407,21 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026-04-10T20:56:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Apr 10, 2026 10:32 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>96</v>
+        <v>273</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -5339,21 +5437,21 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T21:04:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:34 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>30</v>
+        <v>273</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -5364,26 +5462,26 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T19:11:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 7:13 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>2</v>
+        <v>273</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -5399,21 +5497,21 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T18:04:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:35 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>211</v>
+        <v>273</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -5424,26 +5522,26 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:10:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>2</v>
+        <v>242</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -5454,26 +5552,26 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:09:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>3</v>
+        <v>242</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -5489,12 +5587,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07T18:03:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Apr 07, 2026 7:21 PM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -5503,7 +5601,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>78</v>
+        <v>17272</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -5514,26 +5612,26 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>50</v>
+        <v>17272</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -5549,21 +5647,21 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>50</v>
+        <v>1187</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -5579,25 +5677,25 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>203</v>
+        <v>1187</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5609,25 +5707,25 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>203</v>
+        <v>4284</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5639,85 +5737,85 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>150</v>
+        <v>4284</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-16T14:28:00Z</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 16, 2026 2:38 PM GMT</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-16T14:26:00Z</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 16, 2026 2:36 PM GMT</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>123</v>
+        <v>10</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5729,25 +5827,25 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-10T20:56:00Z</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 10, 2026 10:32 PM GMT</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5759,55 +5857,55 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-09T21:04:00Z</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 09, 2026 9:34 PM GMT</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>123</v>
+        <v>30</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-04-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Apr 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>123</v>
+        <v>2</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5819,145 +5917,145 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T21:04:00Z</t>
+          <t>2026-04-09T18:04:00Z</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 10:34 PM GMT</t>
+          <t>Apr 09, 2026 9:35 PM GMT</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>90</v>
+        <v>211</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T17:44:00Z</t>
+          <t>2026-04-08T04:10:00Z</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 6:26 PM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-04-08T04:09:00Z</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-04-07T18:03:00Z</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Apr 07, 2026 7:21 PM GMT</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T00:43:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 12:46 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5969,25 +6067,25 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5999,21 +6097,21 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
@@ -6024,26 +6122,26 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T19:46:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Mar 17, 2026 7:48 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2</v>
+        <v>203</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
@@ -6054,26 +6152,26 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-03-13T00:37:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Mar 13, 2026 12:41 AM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
@@ -6084,26 +6182,26 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2026-03-11T23:50:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Mar 11, 2026 11:54 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
@@ -6119,21 +6217,21 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>164</v>
+        <v>123</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
@@ -6149,21 +6247,21 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>164</v>
+        <v>123</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
@@ -6179,21 +6277,21 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
@@ -6209,21 +6307,21 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
@@ -6239,21 +6337,21 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-20T21:04:00Z</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 20, 2026 10:34 PM GMT</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
@@ -6269,21 +6367,21 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-20T17:44:00Z</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 20, 2026 6:26 PM GMT</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
@@ -6299,21 +6397,21 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
@@ -6329,21 +6427,21 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
@@ -6354,26 +6452,26 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-18T00:43:00Z</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 18, 2026 12:46 AM GMT</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
@@ -6389,21 +6487,21 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>95</v>
+        <v>198</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
@@ -6414,26 +6512,26 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 5:02 PM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>11</v>
+        <v>198</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
@@ -6449,21 +6547,21 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-17T19:46:00Z</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 4:56 PM GMT</t>
+          <t>Mar 17, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
@@ -6479,21 +6577,21 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:44:00Z</t>
+          <t>2026-03-13T00:37:00Z</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 3:15 PM GMT</t>
+          <t>Mar 13, 2026 12:41 AM GMT</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
@@ -6509,21 +6607,21 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:42:00Z</t>
+          <t>2026-03-11T23:50:00Z</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:44 PM GMT</t>
+          <t>Mar 11, 2026 11:54 PM GMT</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
@@ -6534,26 +6632,26 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:41:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:42 PM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
@@ -6564,30 +6662,30 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>2026-02-26T16:39:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Feb 26, 2026 4:44 PM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>5</v>
+        <v>164</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6599,25 +6697,25 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>207</v>
+        <v>85</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6629,25 +6727,25 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>207</v>
+        <v>85</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6659,25 +6757,25 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>159</v>
+        <v>87</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6689,85 +6787,85 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>159</v>
+        <v>87</v>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>2026-02-15T19:46:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Feb 15, 2026 7:48 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14T22:07:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Feb 14, 2026 10:09 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6779,12 +6877,12 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -6793,11 +6891,11 @@
         </is>
       </c>
       <c r="E71" s="5" t="n">
-        <v>282</v>
+        <v>95</v>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
@@ -6809,12 +6907,12 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -6823,88 +6921,88 @@
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>282</v>
+        <v>95</v>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Mar 02, 2026 5:02 PM GMT</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Mar 02, 2026 4:56 PM GMT</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>127</v>
+        <v>5</v>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-03-02T14:44:00Z</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Mar 02, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
@@ -6913,28 +7011,28 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-03-02T14:42:00Z</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Mar 02, 2026 2:44 PM GMT</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -6943,67 +7041,67 @@
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-03-02T14:41:00Z</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Mar 02, 2026 2:42 PM GMT</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-26T16:39:00Z</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 26, 2026 4:44 PM GMT</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -7019,25 +7117,25 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>4234</v>
+        <v>207</v>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7049,145 +7147,145 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>4234</v>
+        <v>207</v>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:46:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:47 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>1</v>
+        <v>159</v>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:45:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:46 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>1</v>
+        <v>159</v>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-02-15T19:46:00Z</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 15, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>1595</v>
+        <v>2</v>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-02-14T22:07:00Z</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 14, 2026 10:09 PM GMT</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E84" s="5" t="n">
-        <v>1595</v>
+        <v>2</v>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7199,55 +7297,55 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T16:24:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Jan 20, 2026 3:26 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>4982</v>
+        <v>282</v>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T15:14:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:15 PM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>1</v>
+        <v>282</v>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7259,85 +7357,85 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T21:13:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:03 PM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>1070</v>
+        <v>127</v>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T04:24:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Jan 15, 2026 4:25 AM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand - Vulncat</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>1</v>
+        <v>127</v>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>2026-01-10T15:08:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Jan 10, 2026 3:10 PM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7349,25 +7447,25 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7379,25 +7477,25 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>140</v>
+        <v>88</v>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7409,25 +7507,25 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E92" s="5" t="n">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -7439,21 +7537,21 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>137</v>
+        <v>4234</v>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
@@ -7469,21 +7567,21 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T00:24:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 1:02 AM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E94" s="5" t="n">
-        <v>38</v>
+        <v>4234</v>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
@@ -7494,37 +7592,457 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-27T14:46:00Z</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Jan 27, 2026 2:47 PM GMT</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-27T14:45:00Z</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Jan 27, 2026 2:46 PM GMT</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="B95" s="5" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-23T23:57:00Z</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="n">
+        <v>1595</v>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-23T23:57:00Z</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - AMS</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="n">
+        <v>1595</v>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-16T16:24:00Z</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Jan 20, 2026 3:26 AM GMT</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="n">
+        <v>4982</v>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-16T15:14:00Z</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Jan 16, 2026 3:15 PM GMT</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-15T21:13:00Z</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Jan 16, 2026 3:03 PM GMT</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>SAST Aviator / ams-sast-aviator</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-15T04:24:00Z</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Jan 15, 2026 4:25 AM GMT</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand - Vulncat</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Outage</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-10T15:08:00Z</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Jan 10, 2026 3:10 PM GMT</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>SAST Aviator / eu-sast-aviator</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T04:54:00Z</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T04:54:00Z</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - AMS</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
         <is>
           <t>2026-01-08T00:24:00Z</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
+      <c r="C108" s="5" t="inlineStr">
         <is>
           <t>Jan 08, 2026 1:02 AM GMT</t>
         </is>
       </c>
-      <c r="D95" s="5" t="inlineStr">
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T00:24:00Z</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 1:02 AM GMT</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
         <is>
           <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
-      <c r="E95" s="5" t="n">
+      <c r="E109" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="F95" s="5" t="inlineStr">
+      <c r="F109" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="11" t="inlineStr">
-        <is>
-          <t>Report revised: May 02, 2026</t>
+    <row r="110">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>Report revised: May 16, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>